<commit_message>
guard: autosave 2026-09-09 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-08 09:30</t>
+          <t>생성: 2026-09-09 08:00</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY674"/>
+  <dimension ref="A1:AY676"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64262,6 +64262,194 @@
       </c>
       <c r="AN674" s="8" t="n">
         <v>876</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B675" s="8" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="C675" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D675" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E675" s="7" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="F675" s="8" t="n">
+        <v>870</v>
+      </c>
+      <c r="G675" s="7" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="H675" s="7" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="I675" s="7" t="n">
+        <v>-12.8</v>
+      </c>
+      <c r="J675" s="7" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="K675" s="7" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="L675" s="7" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="M675" s="7" t="n">
+        <v>-12.8</v>
+      </c>
+      <c r="N675" s="8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="O675" s="8" t="n">
+        <v>271</v>
+      </c>
+      <c r="P675" s="8" t="n">
+        <v>1120</v>
+      </c>
+      <c r="Q675" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R675" s="8" t="n">
+        <v>1114</v>
+      </c>
+      <c r="S675" s="8" t="n">
+        <v>1075</v>
+      </c>
+      <c r="T675" s="8" t="n">
+        <v>1032</v>
+      </c>
+      <c r="U675" s="8" t="n">
+        <v>1070</v>
+      </c>
+      <c r="V675" s="8" t="n">
+        <v>201</v>
+      </c>
+      <c r="W675" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="X675" s="8" t="n">
+        <v>1055</v>
+      </c>
+      <c r="Y675" s="8" t="n">
+        <v>770</v>
+      </c>
+      <c r="Z675" s="8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="AD675" s="8" t="n">
+        <v>2486</v>
+      </c>
+      <c r="AE675" s="8" t="n">
+        <v>1323</v>
+      </c>
+      <c r="AM675" s="8" t="n">
+        <v>1132</v>
+      </c>
+      <c r="AN675" s="8" t="n">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B676" s="8" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="C676" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D676" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E676" s="7" t="n">
+        <v>93</v>
+      </c>
+      <c r="F676" s="8" t="n">
+        <v>895</v>
+      </c>
+      <c r="G676" s="7" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="H676" s="7" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="I676" s="7" t="n">
+        <v>-14.5</v>
+      </c>
+      <c r="J676" s="7" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="K676" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="L676" s="7" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="M676" s="7" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="N676" s="8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="O676" s="8" t="n">
+        <v>246</v>
+      </c>
+      <c r="P676" s="8" t="n">
+        <v>1130</v>
+      </c>
+      <c r="Q676" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R676" s="8" t="n">
+        <v>1147</v>
+      </c>
+      <c r="S676" s="8" t="n">
+        <v>1106</v>
+      </c>
+      <c r="T676" s="8" t="n">
+        <v>1096</v>
+      </c>
+      <c r="U676" s="8" t="n">
+        <v>1070</v>
+      </c>
+      <c r="V676" s="8" t="n">
+        <v>176</v>
+      </c>
+      <c r="W676" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="X676" s="8" t="n">
+        <v>1055</v>
+      </c>
+      <c r="Y676" s="8" t="n">
+        <v>745</v>
+      </c>
+      <c r="Z676" s="8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="AD676" s="8" t="n">
+        <v>2541</v>
+      </c>
+      <c r="AE676" s="8" t="n">
+        <v>1350</v>
+      </c>
+      <c r="AM676" s="8" t="n">
+        <v>1213</v>
+      </c>
+      <c r="AN676" s="8" t="n">
+        <v>929</v>
       </c>
     </row>
   </sheetData>

</xml_diff>